<commit_message>
review and validation of output
</commit_message>
<xml_diff>
--- a/output/saved_column_review.xlsx
+++ b/output/saved_column_review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saved Column Review" sheetId="1" r:id="Rc53441247c214a26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object Index" sheetId="2" r:id="R31fd59926bbc44ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saved Column Review" sheetId="1" r:id="R1e2db560e12040cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object Index" sheetId="2" r:id="R44e97a5272c64fb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1554,7 +1554,7 @@
       </x:c>
       <x:c r="B41" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Portfolio Library Unit"."Library Name"X_Do_Not_Use_</x:t>
+          <x:t xml:space="preserve">"Portfolio Library Unit"."Library Name" is equal to / is in X_Do_Not_Use_</x:t>
         </x:is>
       </x:c>
       <x:c r="C41" s="9" t="inlineStr">
@@ -3150,7 +3150,7 @@
       </x:c>
       <x:c r="B98" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"UNASSIGNEDah92ah9edrrzsea9rqc9mqn9cmuvesx</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in UNASSIGNED; ah92; ah9e; drr; zs; ea9r; qc9m; qn9c; muv; esx</x:t>
         </x:is>
       </x:c>
       <x:c r="C98" s="9" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </x:c>
       <x:c r="B99" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"buchsma9fma9eev9tgsmtsmf9fmf9emfmfsso9fso9e</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in bu; chs; ma9f; ma9e; ev9t; gs; mts; mf9f; mf9e; mf; mfs; so9f; so9e</x:t>
         </x:is>
       </x:c>
       <x:c r="C99" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </x:c>
       <x:c r="B101" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"OUT_RS_REQIN_RS_REQ</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in OUT_RS_REQ; IN_RS_REQ</x:t>
         </x:is>
       </x:c>
       <x:c r="C101" s="9" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </x:c>
       <x:c r="B102" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"anahah9tahuah9aah9lah9dah95ah9gah9jtbtb2tbotb9utb9otb9ptb95tb94tbrtbwtbvtptutuotu94bibicbi9cbifbilbimbi9bbinbbikbirbisbi9dbucbuschchcchnbchpchrdrmamacucbearszweses93es9cesies9mes9bes9dessesweaeaoeateaueaveareaseaxea9wenen9cencen9iensenspevevrevpev2evpoevoevuevsqaqcqclqeqe9fqnqn9kqn9migigrigsititeitiithitpitslblb9lmtmtpmtamcmomo9amo9fmogamo9gmo9mmo9nmo9pmo9ymo9smo9tmumu9mmu9xmucmu9cmuomu9fdnnbqarnbtbrnbtnrnntnrnbqcrnbqernbearnbevrnbcernbitrnbmarnbmnrnbmcrnbmurnbqnrnnclnpuprnbannbahnbbinbbunbchnbesnbeanbennbevnbignbitnblwnbmanbmtnbmunbdnnbphnbsonbssnddondhendlandphndshnlxxnrxxnsxxncmhncmencscnfgenuclnu03unuhtnu01unu02unu03bnu01bnu02bnbphrnbturndsprnlyrrncsprnfsprphpphssososesnbes97eanbeaobennbnbbirnbchrnbdnrndag</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in an; ah; ah9t; ahu; ah9a; ah9l; ah9d; ah95; ah9g; ah9j; tb; tb2; tbo; tb9u; tb9o; tb9p; tb95; tb94; tbr; tbw; tbv; tp; tu; tuo; tu94; bi; bic; bi9c; bif; bil; bim; bi9b; binb; bik; bir; bis; bi9d; buc; bus; ch; chc; chnb; chp; chr; dr; ma; mac; ucbears; zw; es; es93; es9c; esi; es9m; es9b; es9d; ess; esw; ea; eao; eat; eau; eav; ear; eas; eax; ea9w; en; en9c; enc; en9i; ens; ensp; ev; evr; evp; ev2; evpo; evo; evu; evs; qa; qc; qcl; qe; qe9f; qn; qn9k; qn9m; ig; igr; igs; it; ite; iti; ith; itp; its; lb; lb9l; mt; mtp; mta; mc; mo; mo9a; mo9f; moga; mo9g; mo9m; mo9n; mo9p; mo9y; mo9s; mo9t; mu; mu9m; mu9x; muc; mu9c; muo; mu9f; dn; nbqar; nbtbr; nbtnr; nntnr; nbqcr; nbqer; nbear; nbevr; nbcer; nbitr; nbmar; nbmnr; nbmcr; nbmur; nbqnr; nncl; npupr; nban; nbah; nbbi; nbbu; nbch; nbes; nbea; nben; nbev; nbig; nbit; nblw; nbma; nbmt; nbmu; nbdn; nbph; nbso; nbss; nddo; ndhe; ndla; ndph; ndsh; nlxx; nrxx; nsxx; ncmh; ncme; ncsc; nfge; nucl; nu03u; nuht; nu01u; nu02u; nu03b; nu01b; nu02b; nbphr; nbtur; ndspr; nlyrr; ncspr; nfspr; php; phs; so; sos; esnb; es97; eanb; eaob; ennb; nbbir; nbchr; nbdnr; ndag</x:t>
         </x:is>
       </x:c>
       <x:c r="C102" s="9" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </x:c>
       <x:c r="B104" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Executive/ManagementFaculty/Academic StaffGTU FacultyGTU Staff/Visiting ScholarHoward Hughes InstituteLBNL Academic StaffMathematical Sciences Research InstituteProxy - FacultyStanford FacultyUC Extension FacultyUCB Academic Dept Affiliate No ProxyUCB Post-docUCB Visiting Scholar</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Executive/Management; Faculty/Academic Staff; GTU Faculty; GTU Staff/Visiting Scholar; Howard Hughes Institute; LBNL Academic Staff; Mathematical Sciences Research Institute; Proxy - Faculty; Stanford Faculty; UC Extension Faculty; UCB Academic Dept Affiliate No Proxy; UCB Post-doc; UCB Visiting Scholar</x:t>
         </x:is>
       </x:c>
       <x:c r="C104" s="9" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </x:c>
       <x:c r="B105" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Graduate StudentGTU Graduate StudentStanford Graduate Student</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Graduate Student; GTU Graduate Student; Stanford Graduate Student</x:t>
         </x:is>
       </x:c>
       <x:c r="C105" s="9" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </x:c>
       <x:c r="B106" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"LBNL Guest/Temp/ContractorLBNL Non-Academic/Post-docLBNL Retired StaffLibrary Departmental CardLibrary DevelopmentLibrary Retired StaffLibrary StaffLLNL Academic StaffLLNL Non-Academic Staff/Post-docLLNL Retired StaffNon-Academic Retired StaffNon-Academic StaffOther UC RetireeUC Office of the President</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in LBNL Guest/Temp/Contractor; LBNL Non-Academic/Post-doc; LBNL Retired Staff; Library Departmental Card; Library Development; Library Retired Staff; Library Staff; LLNL Academic Staff; LLNL Non-Academic Staff/Post-doc; LLNL Retired Staff; Non-Academic Retired Staff; Non-Academic Staff; Other UC Retiree; UC Office of the President</x:t>
         </x:is>
       </x:c>
       <x:c r="C106" s="9" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </x:c>
       <x:c r="B107" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UC Extension StudentUC Extension Student Non-concurrentUndergraduateUndergraduate - UCB SLE</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UC Extension Student; UC Extension Student Non-concurrent; Undergraduate; Undergraduate - UCB SLE</x:t>
         </x:is>
       </x:c>
       <x:c r="C107" s="9" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </x:c>
       <x:c r="B108" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"AlumniAlumni LifetimeBotanical Garden DocentFaculty/Academic SpouseFaculty/Academic Staff ChildrenInstitute for Historical StudyNon-Academic Staff SpouseReference Use OnlyUCB Academic Dept AffiliateUCB Alumni Association Staff</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Alumni; Alumni Lifetime; Botanical Garden Docent; Faculty/Academic Spouse; Faculty/Academic Staff Children; Institute for Historical Study; Non-Academic Staff Spouse; Reference Use Only; UCB Academic Dept Affiliate; UCB Alumni Association Staff</x:t>
         </x:is>
       </x:c>
       <x:c r="C108" s="9" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </x:c>
       <x:c r="B109" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"CA Private Univ/Coll StudentCA Public School TeachersCA ResidentCA University/Colleges FacultyCA University/Colleges StudentLibrary Non-Affiliated UsersOther UC SpouseCA Private School TeachersDept of Health Services (DHS)ICSI_MSRILibrary Volunteer</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in CA Private Univ/Coll Student; CA Public School Teachers; CA Resident; CA University/Colleges Faculty; CA University/Colleges Student; Library Non-Affiliated Users; Other UC Spouse; CA Private School Teachers; Dept of Health Services (DHS); ICSI_MSRI; Library Volunteer</x:t>
         </x:is>
       </x:c>
       <x:c r="C109" s="9" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </x:c>
       <x:c r="B110" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NETWORKNetwork</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in NETWORK; Network</x:t>
         </x:is>
       </x:c>
       <x:c r="C110" s="9" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </x:c>
       <x:c r="B111" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"ILL Other LibrariesILL UC</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in ILL Other Libraries; ILL UC</x:t>
         </x:is>
       </x:c>
       <x:c r="C111" s="9" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </x:c>
       <x:c r="B113" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"SLF-N Departmental CardSLF-N/UCB Google CartTest Patron GraduateTest Patron UndergraduateNRLF Departmental CardNRLF/UCB Google Cart</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in SLF-N Departmental Card; SLF-N/UCB Google Cart; Test Patron Graduate; Test Patron Undergraduate; NRLF Departmental Card; NRLF/UCB Google Cart</x:t>
         </x:is>
       </x:c>
       <x:c r="C113" s="9" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </x:c>
       <x:c r="B117" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"ILLOUT_RS_REQ</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in ILL; OUT_RS_REQ</x:t>
         </x:is>
       </x:c>
       <x:c r="C117" s="9" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </x:c>
       <x:c r="B119" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"RLISTRESVTPREPCRESRFRESRESSERES</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in RLIST; RESV; TPREP; CRES; RFRES; RES; SERES</x:t>
         </x:is>
       </x:c>
       <x:c r="C119" s="9" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </x:c>
       <x:c r="B120" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"BIOETBMLEXGAMESGENGRESVNEWREFARCHVMRRMLKMEDIAPOPSTXSARESSHLDSBIOVCAMPUSEALEALRFGVMEDGVSTXMANNSHREMMICROOVERASCUCDGROWNPSELRARESPCOLSUPSDEALOVGENSP</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in BIOET; BMLEX; GAMES; GEN; GRESV; NEW; REF; ARCHV; MRR; MLK; MEDIA; POP; STX; SARES; SHLDS; BIOV; CAMPUS; EAL; EALRF; GVMED; GVSTX; MANNSHREM; MICRO; OVER; ASC; UCDGROWN; PSEL; RARE; SPCOL; SUPSD; EALOV; GENSP</x:t>
         </x:is>
       </x:c>
       <x:c r="C120" s="9" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </x:c>
       <x:c r="B122" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Faculty and StaffLaw FacultyUC Ac.Sen., Ac.Fed. &amp; Clin.Fac.(active &amp; retired)UC Research (active &amp; retired)UCD Ac.Sen., Ac.Fed. &amp; Clin.Fac.(active &amp; retired)UCD Research (active &amp; retired)</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Faculty and Staff; Law Faculty; UC Ac.Sen., Ac.Fed. &amp; Clin.Fac.(active &amp; retired); UC Research (active &amp; retired); UCD Ac.Sen., Ac.Fed. &amp; Clin.Fac.(active &amp; retired); UCD Research (active &amp; retired)</x:t>
         </x:is>
       </x:c>
       <x:c r="C122" s="9" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </x:c>
       <x:c r="B123" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Graduate StudentsHealth Sciences Graduate StudentsHealth Sciences ResidentsLaw Students and StaffUC GraduateUCD GraduateUCD Health Sciences GraduateUCD Health Sciences Resident</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Graduate Students; Health Sciences Graduate Students; Health Sciences Residents; Law Students and Staff; UC Graduate; UCD Graduate; UCD Health Sciences Graduate; UCD Health Sciences Resident</x:t>
         </x:is>
       </x:c>
       <x:c r="C123" s="9" t="inlineStr">
@@ -3878,7 +3878,7 @@
       </x:c>
       <x:c r="B124" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Library InternalLibrary Internal - Long LoanInternal Library StaffInternal Library Staff -- In-house useUC Staff (active &amp; retired)UCD Staff (active &amp; retired)</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Library Internal; Library Internal - Long Loan; Internal Library Staff; Internal Library Staff -- In-house use; UC Staff (active &amp; retired); UCD Staff (active &amp; retired)</x:t>
         </x:is>
       </x:c>
       <x:c r="C124" s="9" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </x:c>
       <x:c r="B125" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Undergraduate studentsSpecial UNEX StudentUC UndergraduateUCD Honors Undergraduate (UCD only)</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Undergraduate students; Special UNEX Student; UC Undergraduate; UCD Honors Undergraduate (UCD only)</x:t>
         </x:is>
       </x:c>
       <x:c r="C125" s="9" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </x:c>
       <x:c r="B126" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"MiscellaneousCA college studentsCourtesy -- AlumniCourtesy 10 limitCourtesy 50 limitFee 5 limitProblem patronsStanfordSuspended AccountTemporary AffiliatesUCD Spouse or Adult Child</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Miscellaneous; CA college students; Courtesy -- Alumni; Courtesy 10 limit; Courtesy 50 limit; Fee 5 limit; Problem patrons; Stanford; Suspended Account; Temporary Affiliates; UCD Spouse or Adult Child</x:t>
         </x:is>
       </x:c>
       <x:c r="C126" s="9" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </x:c>
       <x:c r="B127" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Alumni and CA CommunityLaw Visiting ScholarsLaw Public</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Alumni and CA Community; Law Visiting Scholars; Law Public</x:t>
         </x:is>
       </x:c>
       <x:c r="C127" s="9" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </x:c>
       <x:c r="B129" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCD UndergraduateTestzPurge Health Sciences Residents (only assign for Purge Job)zPurge Miscellaneous (only assign for Purge Job)</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCD Undergraduate; Test; zPurge Health Sciences Residents (only assign for Purge Job); zPurge Miscellaneous (only assign for Purge Job)</x:t>
         </x:is>
       </x:c>
       <x:c r="C129" s="9" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </x:c>
       <x:c r="B131" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Interlibrary LoanInterlibrary Loan -- UC Fac/Grad</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Interlibrary Loan; Interlibrary Loan -- UC Fac/Grad</x:t>
         </x:is>
       </x:c>
       <x:c r="C131" s="9" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </x:c>
       <x:c r="B135" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"UNASSIGNEDsrlf</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in UNASSIGNED; srlf</x:t>
         </x:is>
       </x:c>
       <x:c r="C135" s="9" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </x:c>
       <x:c r="B136" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"gmlmlxllexllckxllhkxeqsaxslkbxslexslkd</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in gmlml; xlle; xllck; xllhk; xeqsa; xslkb; xsle; xslkd</x:t>
         </x:is>
       </x:c>
       <x:c r="C136" s="9" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </x:c>
       <x:c r="B137" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"gmlilllawillllill_rsllawill_rslslill</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in gmlill; lawill; llill_rsl; lawill_rsl; slill</x:t>
         </x:is>
       </x:c>
       <x:c r="C137" s="9" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </x:c>
       <x:c r="B138" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"gmlresllreslawcrslrespermslresslresmedia</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in gmlres; llres; lawcr; slresperm; slres; slresmedia</x:t>
         </x:is>
       </x:c>
       <x:c r="C138" s="9" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </x:c>
       <x:c r="B139" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"gmlgseadgocrhgseaallllxllcomlldoseacoleaoseanbgpcagploceakorllldllcppllmicllloblllobillosllbprllpullreflltoslawcslawfdlawrrlawreflawreslawstackslawsupslslbgsldosgpusslmediaslrefmediaslvaultslosllcprearefllledspcollawcd</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in gml; gsead; gocrh; gseaa; ll; llx; llcom; lldos; eacol; eaos; eanb; gpca; gploc; eakor; llld; llcpp; llmic; lllob; lllobi; llos; llbpr; llpu; llref; lltos; lawcs; lawfd; lawrr; lawref; lawres; lawstacks; lawsup; sl; slbg; sldos; gpus; slmedia; slrefmedia; slvault; slos; llcpr; earef; llled; spcol; lawcd</x:t>
         </x:is>
       </x:c>
       <x:c r="C139" s="9" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </x:c>
       <x:c r="B141" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCI Arts FacultyUCI FacultyUCI Faculty DDSUCI Law FacultyUCI LibrarianUCI Arts Faculty DDSUCI Division of Continuing Education FacultyVisiting Scholar</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCI Arts Faculty; UCI Faculty; UCI Faculty DDS; UCI Law Faculty; UCI Librarian; UCI Arts Faculty DDS; UCI Division of Continuing Education Faculty; Visiting Scholar</x:t>
         </x:is>
       </x:c>
       <x:c r="C141" s="9" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </x:c>
       <x:c r="B142" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCI Graduate StudentUCI Law Graduate StudentUCI Law JournalUCI Graduate Student DDS</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCI Graduate Student; UCI Law Graduate Student; UCI Law Journal; UCI Graduate Student DDS</x:t>
         </x:is>
       </x:c>
       <x:c r="C142" s="9" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </x:c>
       <x:c r="B143" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCI Law StaffUCI Law Staff DDSUCI Library StaffUCI Retired StaffUCI StaffUCI Staff DDS</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCI Law Staff; UCI Law Staff DDS; UCI Library Staff; UCI Retired Staff; UCI Staff; UCI Staff DDS</x:t>
         </x:is>
       </x:c>
       <x:c r="C143" s="9" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </x:c>
       <x:c r="B144" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCI Division of Continuing Education StudentUCI Honors StudentUCI Regents Scholar/UROPUCI Undergraduate Student</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCI Division of Continuing Education Student; UCI Honors Student; UCI Regents Scholar/UROP; UCI Undergraduate Student</x:t>
         </x:is>
       </x:c>
       <x:c r="C144" s="9" t="inlineStr">
@@ -4466,7 +4466,7 @@
       </x:c>
       <x:c r="B145" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"CommunityCommunity College Honors StudentHigh School Student</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Community; Community College Honors Student; High School Student</x:t>
         </x:is>
       </x:c>
       <x:c r="C145" s="9" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </x:c>
       <x:c r="B146" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Other FacultyOther Graduate StudentOther Undergraduate StudentUCI Law Alumni</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Other Faculty; Other Graduate Student; Other Undergraduate Student; UCI Law Alumni</x:t>
         </x:is>
       </x:c>
       <x:c r="C146" s="9" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </x:c>
       <x:c r="B147" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NetworkUC FacultyILL Lending UC</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Network; UC Faculty; ILL Lending UC</x:t>
         </x:is>
       </x:c>
       <x:c r="C147" s="9" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </x:c>
       <x:c r="B149" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCI Library Department CardPURGE</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCI Library Department Card; PURGE</x:t>
         </x:is>
       </x:c>
       <x:c r="C149" s="9" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </x:c>
       <x:c r="B152" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"5542561600006533arcgabxuechltuerfyrcleanupyrcatsupyrgic</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in 5542561600006533; arcgabx; uechlt; uerf; yrcleanup; yrcatsup; yrgic</x:t>
         </x:is>
       </x:c>
       <x:c r="C152" s="9" t="inlineStr">
@@ -4690,7 +4690,7 @@
       </x:c>
       <x:c r="B153" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"archromearpubcircartcliccbichromebiocliccbipubcircboechromeboecliccboepubcirccccollegeclasscliccclchromeclicclockecliccpnloccliccpsloccliccynloccliccyslocmgpubcircmuchromemusiccliccsgcliccUNASSIGNEDyrchromecliccpkskcliccykskmgchromeclpubcircyrpubcirc</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in archrome; arpubcirc; artclicc; bichrome; bioclicc; bipubcirc; boechrome; boeclicc; boepubcirc; cccollege; classclicc; clchrome; clicclocke; cliccpnloc; cliccpsloc; cliccynloc; cliccysloc; mgpubcirc; muchrome; musicclicc; sgclicc; UNASSIGNED; yrchrome; cliccpksk; cliccyksk; mgchrome; clpubcirc; yrpubcirc</x:t>
         </x:is>
       </x:c>
       <x:c r="C153" s="9" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </x:c>
       <x:c r="B155" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"lwillOUT_RS_REQ</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in lwill; OUT_RS_REQ</x:t>
         </x:is>
       </x:c>
       <x:c r="C155" s="9" t="inlineStr">
@@ -4774,7 +4774,7 @@
       </x:c>
       <x:c r="B156" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"arcrbirsbirsprscpclrsearslwrslwrspermgcirsmgrsmgrsstrgmurssmcrsyrcipryrrs</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in arcr; birs; birsprscp; clrs; ears; lwrs; lwrsper; mgcirs; mgrs; mgrsstrg; murs; smcrs; yrcipr; yrrs</x:t>
         </x:is>
       </x:c>
       <x:c r="C156" s="9" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </x:c>
       <x:c r="B157" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"ararcgarcgabarcgabxxarcgxarcotfarmediaarperarperxarplayarrfarrsarscriptartsTSarxarxx-xxxbibicidpermbicotfbiperbirfbirsclasclclcareerclcookcldispclenigclgrfnclnrfcclofclpermclsustaincltravclvidgamesclzineeaeadiujnleaovereaxeaxxherblsbihilsbirfhistlsyrstaxlwlwcivideolwcixlwcleanuplwofrflwphillwrflwsuperlwtrrlwwilliamsmgcleanupmgnbksmgrfmgsccohimumuclsdmuclsdmmmuclsdsdrmuminimunbksmuxmuxxmuxxxsgsgansgcotfsgdispsgmisgpersgputsmsmavsmcotfsmpersmrspermsmsctallmsrsrarsrar2srbi2srbuosrcasrcksrcrsretsrilsrmnmsrnoncircsrubsruclsrucl2srucl3srucl4srud0srud2srui2srursryr2sryr7sryr8ue123eueabceueaubksuebiogueefolkueestaxueficueficeruefolkueforuenficuepapuepoeuesmalleuesxyryralmiyranyranxyrciyrlcotfyrllostyrmiclsdyrpeyrperyrrisatlyrrisrryrxyrxxyrxxxartsbixcaearfclgamesryr9</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in ar; arcg; arcgab; arcgabxx; arcgx; arcotf; armedia; arper; arperx; arplay; arrf; arrs; arscript; artsTS; arx; arxx-xxx; bi; bicidperm; bicotf; biper; birf; birsclas; cl; clcareer; clcook; cldisp; clenig; clgrfn; clnrfc; clof; clperm; clsustain; cltrav; clvidgames; clzine; ea; eadiujnl; eaover; eax; eaxx; herb; lsbihi; lsbirfhist; lsyrstax; lw; lwcivideo; lwcix; lwcleanup; lwofrf; lwphil; lwrf; lwsuper; lwtrr; lwwilliams; mgcleanup; mgnbks; mgrf; mgsccohi; mu; muclsd; muclsdmm; muclsdsdr; mumini; munbks; mux; muxx; muxxx; sg; sgan; sgcotf; sgdisp; sgmi; sgper; sgput; sm; smav; smcotf; smper; smrsperm; smsctallm; sr; srar; srar2; srbi2; srbuo; srca; srck; srcr; sret; sril; srmnm; srnoncirc; srub; srucl; srucl2; srucl3; srucl4; srud0; srud2; srui2; srur; sryr2; sryr7; sryr8; ue123e; ueabce; ueaubks; uebiog; ueefolk; ueestax; uefic; ueficer; uefolk; uefor; uenfic; uepap; uepoe; uesmalle; uesx; yr; yralmi; yran; yranx; yrci; yrlcotf; yrllost; yrmiclsd; yrpe; yrper; yrrisatl; yrrisrr; yrx; yrxx; yrxxx; arts; bix; ca; earf; clgame; sryr9</x:t>
         </x:is>
       </x:c>
       <x:c r="C157" s="9" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </x:c>
       <x:c r="B159" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCLA Acad - NoLimitUCLA Acad ProxyUCLA AcademicUCLA Law AcademicUCLA Law ProxyUCLA Retired Academic</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCLA Acad - NoLimit; UCLA Acad Proxy; UCLA Academic; UCLA Law Academic; UCLA Law Proxy; UCLA Retired Academic</x:t>
         </x:is>
       </x:c>
       <x:c r="C159" s="9" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </x:c>
       <x:c r="B160" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCLA GraduateUCLA Law GradUCLA Mgmt PhDUCLA Music GradUCLA Grad NoLimit</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCLA Graduate; UCLA Law Grad; UCLA Mgmt PhD; UCLA Music Grad; UCLA Grad NoLimit</x:t>
         </x:is>
       </x:c>
       <x:c r="C160" s="9" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </x:c>
       <x:c r="B161" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Internal Use OnlyUCLA Law StaffUCLA Lib Staff RecallUCLA Staff</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Internal Use Only; UCLA Law Staff; UCLA Lib Staff Recall; UCLA Staff</x:t>
         </x:is>
       </x:c>
       <x:c r="C161" s="9" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </x:c>
       <x:c r="B162" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCLA Music UndergradUCLA Undergrad</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCLA Music Undergrad; UCLA Undergrad</x:t>
         </x:is>
       </x:c>
       <x:c r="C162" s="9" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </x:c>
       <x:c r="B163" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Early ChildhoodExtensionExternal 10 - AssociatesExternal 10 - UCLA AlumniGeffen Academy StudentLab School ParentLab School StudentSPRUCLA Retired StaffVGR</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Early Childhood; Extension; External 10 - Associates; External 10 - UCLA Alumni; Geffen Academy Student; Lab School Parent; Lab School Student; SPR; UCLA Retired Staff; VGR</x:t>
         </x:is>
       </x:c>
       <x:c r="C163" s="9" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </x:c>
       <x:c r="B164" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Access OnlyAP/TAP StudentExternal 10External 20External 200 - FacultyExternal 200 - OtherExternal 5 - OtherExternal 50 - Corporation</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Access Only; AP/TAP Student; External 10; External 20; External 200 - Faculty; External 200 - Other; External 5 - Other; External 50 - Corporation</x:t>
         </x:is>
       </x:c>
       <x:c r="C164" s="9" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </x:c>
       <x:c r="B165" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NETWORKNetwork</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in NETWORK; Network</x:t>
         </x:is>
       </x:c>
       <x:c r="C165" s="9" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </x:c>
       <x:c r="B166" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"ILL Department - Non UCILL Department - UC</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in ILL Department - Non UC; ILL Department - UC</x:t>
         </x:is>
       </x:c>
       <x:c r="C166" s="9" t="inlineStr">
@@ -5110,7 +5110,7 @@
       </x:c>
       <x:c r="B168" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"EHSUCLA Library Staff DepartmentUsers to Purge</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in EHS; UCLA Library Staff Department; Users to Purge</x:t>
         </x:is>
       </x:c>
       <x:c r="C168" s="9" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </x:c>
       <x:c r="B173" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"disgenSvcs DeskspcUNASSIGNEDHold</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in dis; gen; Svcs Desk; spc; UNASSIGNED; Hold</x:t>
         </x:is>
       </x:c>
       <x:c r="C173" s="9" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </x:c>
       <x:c r="B177" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Library StaffUCM Staff</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Library Staff; UCM Staff</x:t>
         </x:is>
       </x:c>
       <x:c r="C177" s="9" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </x:c>
       <x:c r="B180" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"CA Community College StudentFee AccountUC Alumni Association MemberCA Public School Employee</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in CA Community College Student; Fee Account; UC Alumni Association Member; CA Public School Employee</x:t>
         </x:is>
       </x:c>
       <x:c r="C180" s="9" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </x:c>
       <x:c r="B181" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NetworkNETWORK</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Network; NETWORK</x:t>
         </x:is>
       </x:c>
       <x:c r="C181" s="9" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </x:c>
       <x:c r="B187" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"srlfSRLF</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in srlf; SRLF</x:t>
         </x:is>
       </x:c>
       <x:c r="C187" s="9" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </x:c>
       <x:c r="B189" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"orbcircorbcmorbneworbpopsciorbreforbstacksorboverwrcaorbshelfnoorbwrcacirccdwrcastacksedcurricedhangingedjuvenileedjuvtinyedmiscedoversizeedtextbookgovcagovpamusgovusrivleisurerivmobyrivcircrivcmrivinfodskrivmedblryrivmediacdrivmedcmflrivmeddvdrivmedrecdrivmedvhsrivmedvdgmrivmfilmrivnewrivrefrivstacksrivflatrivoverrivstyscwrcarivshelfclosesrlfpenrivorbflatwrcacircedjuvbigexhibit1govsmfichesrlfpendwrcamcase</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in orbcirc; orbcm; orbnew; orbpopsci; orbref; orbstacks; orbover; wrcaorb; shelfnoorb; wrcacirccd; wrcastacks; edcurric; edhanging; edjuvenile; edjuvtiny; edmisc; edoversize; edtextbook; govca; govpamus; govus; rivleisure; rivmoby; rivcirc; rivcm; rivinfodsk; rivmedblry; rivmediacd; rivmedcmfl; rivmeddvd; rivmedrecd; rivmedvhs; rivmedvdgm; rivmfilm; rivnew; rivref; rivstacks; rivflat; rivover; rivstysc; wrcariv; shelfclose; srlfpenriv; orbflat; wrcacirc; edjuvbig; exhibit1; govsmfiche; srlfpend; wrcamcase</x:t>
         </x:is>
       </x:c>
       <x:c r="C189" s="9" t="inlineStr">
@@ -5754,7 +5754,7 @@
       </x:c>
       <x:c r="B191" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Emeritus FacultyUCR AcademicUCR Library StaffProxy</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Emeritus Faculty; UCR Academic; UCR Library Staff; Proxy</x:t>
         </x:is>
       </x:c>
       <x:c r="C191" s="9" t="inlineStr">
@@ -5810,7 +5810,7 @@
       </x:c>
       <x:c r="B193" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Retired StaffUCR StaffInternal Use - Reserves Instructor</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Retired Staff; UCR Staff; Internal Use - Reserves Instructor</x:t>
         </x:is>
       </x:c>
       <x:c r="C193" s="9" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </x:c>
       <x:c r="B194" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Concurrent EnrollmentUCR Undergraduate</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Concurrent Enrollment; UCR Undergraduate</x:t>
         </x:is>
       </x:c>
       <x:c r="C194" s="9" t="inlineStr">
@@ -5866,7 +5866,7 @@
       </x:c>
       <x:c r="B195" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UCR AlumniUCR ExtensionCourtesy - UCR Extension InstructorVolunteer Clinical Faculty</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UCR Alumni; UCR Extension; Courtesy - UCR Extension Instructor; Volunteer Clinical Faculty</x:t>
         </x:is>
       </x:c>
       <x:c r="C195" s="9" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </x:c>
       <x:c r="B196" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Certificated TeachersCommunity Borrowing CardContractual Agreement - RCC HonorsCourtesy - IB ProgramCourtesy - Spouse/Partner/ChildNon-UC Academic - CSUNon-UC Academic - PrivateNon-UC Academic – Community CollegeProfessional Agreement - CARBProfessional Agreement – Mentor ProgramProfessional Agreement – UnpaidContractual Agreement - Loma LindaContractual Agreement - RedlandsContractual Agreement - StanfordCourtesy - Capstone ProgramCourtesy - PE ReporterProfessional Agreement – USDA Fire LabProfessional Agreement – USDA Salinity LabProfessional Agreement – USDI/GSSpecial – Friends of the CampusSpecial – Independent Scholar</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Certificated Teachers; Community Borrowing Card; Contractual Agreement - RCC Honors; Courtesy - IB Program; Courtesy - Spouse/Partner/Child; Non-UC Academic - CSU; Non-UC Academic - Private; Non-UC Academic – Community College; Professional Agreement - CARB; Professional Agreement – Mentor Program; Professional Agreement – Unpaid; Contractual Agreement - Loma Linda; Contractual Agreement - Redlands; Contractual Agreement - Stanford; Courtesy - Capstone Program; Courtesy - PE Reporter; Professional Agreement – USDA Fire Lab; Professional Agreement – USDA Salinity Lab; Professional Agreement – USDI/GS; Special – Friends of the Campus; Special – Independent Scholar</x:t>
         </x:is>
       </x:c>
       <x:c r="C196" s="9" t="inlineStr">
@@ -5922,7 +5922,7 @@
       </x:c>
       <x:c r="B197" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UC AffiliatesUC Alumni</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UC Affiliates; UC Alumni</x:t>
         </x:is>
       </x:c>
       <x:c r="C197" s="9" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </x:c>
       <x:c r="B199" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Non-UC ILLUC ILLNon-UC Academic - OCLC</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Non-UC ILL; UC ILL; Non-UC Academic - OCLC</x:t>
         </x:is>
       </x:c>
       <x:c r="C199" s="9" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </x:c>
       <x:c r="B202" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"NRLFSRLF</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in NRLF; SRLF</x:t>
         </x:is>
       </x:c>
       <x:c r="C202" s="9" t="inlineStr">
@@ -6202,7 +6202,7 @@
       </x:c>
       <x:c r="B207" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"RBSFCRBS</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in RBSFC; RBS</x:t>
         </x:is>
       </x:c>
       <x:c r="C207" s="9" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </x:c>
       <x:c r="B208" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"EGANARAECARTSAROVEGASEGBLBROWSINGEGCTNMACSCURCURJMASIANASNOVEGWMMILRFGPCAGPLOGPMEDGPUSGPUSOMAINMEDIAMAMFCMAMFMMUSMUDSKMUCDMULPMUVIDMUFOLMUMNIMUOVEGNAART_TEMPMAOVMARFSELSELOVARSJCSHPR-SELARGNCARGCOEGCTOASNBRGPCENCIRC_UNCATSPEC</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in EGAN; ARAEC; ARTS; AROV; EGAS; EGBL; BROWSING; EGCTN; MACS; CUR; CURJM; ASIAN; ASNOV; EGWM; MILRF; GPCA; GPLO; GPMED; GPUS; GPUSO; MAIN; MEDIA; MAMFC; MAMFM; MUS; MUDSK; MUCD; MULP; MUVID; MUFOL; MUMNI; MUOV; EGNA; ART_TEMP; MAOV; MARF; SEL; SELOV; ARSJC; SHPR-SEL; ARGNC; ARGCO; EGCTO; ASNBR; GPCEN; CIRC_UNCAT; SPEC</x:t>
         </x:is>
       </x:c>
       <x:c r="C208" s="9" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </x:c>
       <x:c r="B210" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Faculty, AnnualFaculty, Quarter</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Faculty, Annual; Faculty, Quarter</x:t>
         </x:is>
       </x:c>
       <x:c r="C210" s="9" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </x:c>
       <x:c r="B211" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Student, AnnualStudent, Quarter</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Student, Annual; Student, Quarter</x:t>
         </x:is>
       </x:c>
       <x:c r="C211" s="9" t="inlineStr">
@@ -6398,7 +6398,7 @@
       </x:c>
       <x:c r="B214" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Community, LimitedCourtesy with Journal Privileges</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Community, Limited; Courtesy with Journal Privileges</x:t>
         </x:is>
       </x:c>
       <x:c r="C214" s="9" t="inlineStr">
@@ -6426,7 +6426,7 @@
       </x:c>
       <x:c r="B215" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NETWORKNetwork</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in NETWORK; Network</x:t>
         </x:is>
       </x:c>
       <x:c r="C215" s="9" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </x:c>
       <x:c r="B216" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"DepartmentProxy, AnnualCorporatePremium Community - DO NOT USE</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Department; Proxy, Annual; Corporate; Premium Community - DO NOT USE</x:t>
         </x:is>
       </x:c>
       <x:c r="C216" s="9" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </x:c>
       <x:c r="B221" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"nrlfNRLF</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in nrlf; NRLF</x:t>
         </x:is>
       </x:c>
       <x:c r="C221" s="9" t="inlineStr">
@@ -6622,7 +6622,7 @@
       </x:c>
       <x:c r="B222" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"mheqpmedequipdsisequp</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in mheqp; medequip; dsi; sequp</x:t>
         </x:is>
       </x:c>
       <x:c r="C222" s="9" t="inlineStr">
@@ -6706,7 +6706,7 @@
       </x:c>
       <x:c r="B225" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"mhresmedrescres</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in mhres; medre; scres</x:t>
         </x:is>
       </x:c>
       <x:c r="C225" s="9" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </x:c>
       <x:c r="B226" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"mycurmycovmgcalmgusmprotmrefmrdskmrovrmstaxmstovmformmfgdespcmedccmedmeddoeastsgamescprosreadsstaxsstovmhmedccmhmed</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in mycur; mycov; mgcal; mgus; mprot; mref; mrdsk; mrovr; mstax; mstov; mform; mfgde; spc; medcc; med; meddo; east; sgame; scpro; sread; sstax; sstov; mhmedcc; mhmed</x:t>
         </x:is>
       </x:c>
       <x:c r="C226" s="9" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </x:c>
       <x:c r="B233" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NETWORKNetwork</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in NETWORK; Network</x:t>
         </x:is>
       </x:c>
       <x:c r="C233" s="9" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </x:c>
       <x:c r="B236" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"DefaultEXHIBITSILL LONG-TERM 1ILL LONG-TERM 2ILL SHORT-TERM 1ILL SHORT-TERM 2LIBRARY 1 YEARMEDIA IN HOUSE</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Default; EXHIBITS; ILL LONG-TERM 1; ILL LONG-TERM 2; ILL SHORT-TERM 1; ILL SHORT-TERM 2; LIBRARY 1 YEAR; MEDIA IN HOUSE</x:t>
         </x:is>
       </x:c>
       <x:c r="C236" s="9" t="inlineStr">
@@ -7070,7 +7070,7 @@
       </x:c>
       <x:c r="B238" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"cc_borbotcc_flr2cc_stordesk</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in cc_borbot; cc_flr2; cc_stor; desk</x:t>
         </x:is>
       </x:c>
       <x:c r="C238" s="9" t="inlineStr">
@@ -7126,7 +7126,7 @@
       </x:c>
       <x:c r="B240" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"OUT_CT_REQOUT_RS_REQIN_CT_REQ</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in OUT_CT_REQ; OUT_RS_REQ; IN_CT_REQ</x:t>
         </x:is>
       </x:c>
       <x:c r="C240" s="9" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </x:c>
       <x:c r="B241" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"res_borbotresres_stor</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in res_borbot; res; res_stor</x:t>
         </x:is>
       </x:c>
       <x:c r="C241" s="9" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </x:c>
       <x:c r="B242" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"vid_borbotcc_radbks_fl1bks_fl5bks_fl6bks_fl7bks_fl8calm_cavecc_fl1cc_fl1_ovdoc_cadoc_sddoc_usdoc_us2ea_oveaovx_fl1ovx_fl6gslgis_refgraph_novindexjrnl_fl1bks_popmaps_cabinmeet_spotmicronew_booksov_fl1ov_fl6pop_scirefvideoaudiobksccdissfilmjrnlov</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in vid_borbot; cc_rad; bks_fl1; bks_fl5; bks_fl6; bks_fl7; bks_fl8; calm_cave; cc_fl1; cc_fl1_ov; doc_ca; doc_sd; doc_us; doc_us2; ea_ov; ea; ovx_fl1; ovx_fl6; gsl; gis_ref; graph_nov; index; jrnl_fl1; bks_pop; maps_cabin; meet_spot; micro; new_books; ov_fl1; ov_fl6; pop_sci; ref; video; audio; bks; cc; diss; film; jrnl; ov</x:t>
         </x:is>
       </x:c>
       <x:c r="C242" s="9" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </x:c>
       <x:c r="B244" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Post DocUC AcademicVisiting Scholar</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Post Doc; UC Academic; Visiting Scholar</x:t>
         </x:is>
       </x:c>
       <x:c r="C244" s="9" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </x:c>
       <x:c r="B245" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UC Graduate StudentVisiting Graduate Student</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UC Graduate Student; Visiting Graduate Student</x:t>
         </x:is>
       </x:c>
       <x:c r="C245" s="9" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </x:c>
       <x:c r="B246" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"UC StaffUCSD Library Staff</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in UC Staff; UCSD Library Staff</x:t>
         </x:is>
       </x:c>
       <x:c r="C246" s="9" t="inlineStr">
@@ -7406,7 +7406,7 @@
       </x:c>
       <x:c r="B250" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NETWORKNetwork</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in NETWORK; Network</x:t>
         </x:is>
       </x:c>
       <x:c r="C250" s="9" t="inlineStr">
@@ -7434,7 +7434,7 @@
       </x:c>
       <x:c r="B251" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"Interlibrary LoanInterlibrary Loan - UC</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Interlibrary Loan; Interlibrary Loan - UC</x:t>
         </x:is>
       </x:c>
       <x:c r="C251" s="9" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </x:c>
       <x:c r="B257" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"rbrmbr</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in rbr; mbr</x:t>
         </x:is>
       </x:c>
       <x:c r="C257" s="9" t="inlineStr">
@@ -7630,7 +7630,7 @@
       </x:c>
       <x:c r="B258" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code"mbccb4thflovrszpspopbtpopref</x:t>
+          <x:t xml:space="preserve">"Item Location at Time of Loan"."Location Code" is equal to / is in mbccb; 4thfl; ovrsz; pspop; btpop; ref</x:t>
         </x:is>
       </x:c>
       <x:c r="C258" s="9" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </x:c>
       <x:c r="B263" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Borrower Details"."User Group"NetworkNETWORK</x:t>
+          <x:t xml:space="preserve">"Borrower Details"."User Group" is equal to / is in Network; NETWORK</x:t>
         </x:is>
       </x:c>
       <x:c r="C263" s="9" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </x:c>
       <x:c r="B444" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"zw</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in zw</x:t>
         </x:is>
       </x:c>
       <x:c r="C444" s="9" t="inlineStr">
@@ -13034,7 +13034,7 @@
       </x:c>
       <x:c r="B451" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"ahah9tdldndrgsma9xmfmoss</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in ah; ah9t; dl; dn; dr; gs; ma9x; mf; mo; ss</x:t>
         </x:is>
       </x:c>
       <x:c r="C451" s="9" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </x:c>
       <x:c r="B452" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"tbtj</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in tb; tj</x:t>
         </x:is>
       </x:c>
       <x:c r="C452" s="9" t="inlineStr">
@@ -13118,7 +13118,7 @@
       </x:c>
       <x:c r="B454" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"mt</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in mt</x:t>
         </x:is>
       </x:c>
       <x:c r="C454" s="9" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </x:c>
       <x:c r="B455" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"ma</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in ma</x:t>
         </x:is>
       </x:c>
       <x:c r="C455" s="9" t="inlineStr">
@@ -13174,7 +13174,7 @@
       </x:c>
       <x:c r="B456" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"bu</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in bu</x:t>
         </x:is>
       </x:c>
       <x:c r="C456" s="9" t="inlineStr">
@@ -13202,7 +13202,7 @@
       </x:c>
       <x:c r="B457" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"mu</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in mu</x:t>
         </x:is>
       </x:c>
       <x:c r="C457" s="9" t="inlineStr">
@@ -13230,7 +13230,7 @@
       </x:c>
       <x:c r="B458" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"so</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in so</x:t>
         </x:is>
       </x:c>
       <x:c r="C458" s="9" t="inlineStr">
@@ -13258,7 +13258,7 @@
       </x:c>
       <x:c r="B459" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"ch</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in ch</x:t>
         </x:is>
       </x:c>
       <x:c r="C459" s="9" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </x:c>
       <x:c r="B460" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"an</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in an</x:t>
         </x:is>
       </x:c>
       <x:c r="C460" s="9" t="inlineStr">
@@ -13314,7 +13314,7 @@
       </x:c>
       <x:c r="B461" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"es</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in es</x:t>
         </x:is>
       </x:c>
       <x:c r="C461" s="9" t="inlineStr">
@@ -13342,7 +13342,7 @@
       </x:c>
       <x:c r="B462" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"it</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in it</x:t>
         </x:is>
       </x:c>
       <x:c r="C462" s="9" t="inlineStr">
@@ -13398,7 +13398,7 @@
       </x:c>
       <x:c r="B464" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"oh</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in oh</x:t>
         </x:is>
       </x:c>
       <x:c r="C464" s="9" t="inlineStr">
@@ -13426,7 +13426,7 @@
       </x:c>
       <x:c r="B465" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"mc</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in mc</x:t>
         </x:is>
       </x:c>
       <x:c r="C465" s="9" t="inlineStr">
@@ -13454,7 +13454,7 @@
       </x:c>
       <x:c r="B466" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"ig</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in ig</x:t>
         </x:is>
       </x:c>
       <x:c r="C466" s="9" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </x:c>
       <x:c r="B467" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"qaxqcxqnx</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in qax; qcx; qnx</x:t>
         </x:is>
       </x:c>
       <x:c r="C467" s="9" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </x:c>
       <x:c r="B468" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"lawbwb</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in lawb; wb</x:t>
         </x:is>
       </x:c>
       <x:c r="C468" s="9" t="inlineStr">
@@ -13538,7 +13538,7 @@
       </x:c>
       <x:c r="B469" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"ph</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in ph</x:t>
         </x:is>
       </x:c>
       <x:c r="C469" s="9" t="inlineStr">
@@ -13566,7 +13566,7 @@
       </x:c>
       <x:c r="B470" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"n</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in n</x:t>
         </x:is>
       </x:c>
       <x:c r="C470" s="9" t="inlineStr">
@@ -13594,7 +13594,7 @@
       </x:c>
       <x:c r="B471" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"bi</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in bi</x:t>
         </x:is>
       </x:c>
       <x:c r="C471" s="9" t="inlineStr">
@@ -13622,7 +13622,7 @@
       </x:c>
       <x:c r="B472" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"evce</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in ev; ce</x:t>
         </x:is>
       </x:c>
       <x:c r="C472" s="9" t="inlineStr">
@@ -13650,7 +13650,7 @@
       </x:c>
       <x:c r="B473" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Location"."Location Code"qaqcqeqn</x:t>
+          <x:t xml:space="preserve">"Location"."Location Code" is equal to / is in qa; qc; qe; qn</x:t>
         </x:is>
       </x:c>
       <x:c r="C473" s="9" t="inlineStr">
@@ -14546,7 +14546,7 @@
       </x:c>
       <x:c r="B505" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Electronic Collection"."Electronic Collection Public Name"Ebook Central Perpetual, DDA and Subscription TitlesEBSCO (UCSD). eBook Collection DDA online monographs.R2 Digital Library DDA</x:t>
+          <x:t xml:space="preserve">"Electronic Collection"."Electronic Collection Public Name" is equal to / is in Ebook Central Perpetual, DDA and Subscription Titles; EBSCO (UCSD). eBook Collection DDA online monographs.; R2 Digital Library DDA</x:t>
         </x:is>
       </x:c>
       <x:c r="C505" s="9" t="inlineStr">
@@ -14574,7 +14574,7 @@
       </x:c>
       <x:c r="B506" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">"Electronic Collection"."Electronic Collection Public Name"British and Irish Women's Letters and Diaries: First Edition (Pre-January 2009 Purchasers Only)Books@Ovid - LWW JBIB Book Collection 2017-2018 PurchaseBooks@Ovid PurchaseBooks@Ovid Purchase CompleteNorth American Indian Drama: First Edition (Pre-October 2012 Purchasers Only)Twentieth Century North American Drama: First Edition (Pre-October 2012 Purchasers Only)Institute of Physics Historic Archive PurchaseMaruzen eBook LibraryBerkeley LDC purchasesIGI Global Evidence Based PURCHASEDOxford University Press Anthropology Local Purchased CollectionSage EBSSage online monographs EBS (Sage EBS) purchasedUC Davis locally purchased monographs_LOCALUCSC owned streaming videoAfrican Writers Series (pre-September 2011 purchase)SAGE Complete Deep Backfile Purchase 2008SAGE Deep Backfile Upgrade Purchase 2009SAGE Deep Backfile Upgrade Purchase 2010SAGE Deep Backfile Upgrade Purchase 2011SAGE Deep Backfile Upgrade Purchase 2012SAGE Deep Backfile Upgrade Purchase 2013SAGE Deep Backfile Upgrade Purchase 2014SAGE Deep Backfile Upgrade Purchase 2015SAGE Deep Backfile Upgrade Purchase 2016SAGE Deep Backfile Upgrade Purchase 2017SAGE Psychology Subject Collection Backfile PurchaseTaylor &amp; Francis online monographs (EBS) purchased</x:t>
+          <x:t xml:space="preserve">"Electronic Collection"."Electronic Collection Public Name" is equal to / is in British and Irish Women's Letters and Diaries: First Edition (Pre-January 2009 Purchasers Only); Books@Ovid - LWW JBIB Book Collection 2017-2018 Purchase; Books@Ovid Purchase; Books@Ovid Purchase Complete; North American Indian Drama: First Edition (Pre-October 2012 Purchasers Only); Twentieth Century North American Drama: First Edition (Pre-October 2012 Purchasers Only); Institute of Physics Historic Archive Purchase; Maruzen eBook Library; Berkeley LDC purchases; IGI Global Evidence Based PURCHASED; Oxford University Press Anthropology Local Purchased Collection; Sage EBS; Sage online monographs EBS (Sage EBS) purchased; UC Davis locally purchased monographs_LOCAL; UCSC owned streaming video; African Writers Series (pre-September 2011 purchase); SAGE Complete Deep Backfile Purchase 2008; SAGE Deep Backfile Upgrade Purchase 2009; SAGE Deep Backfile Upgrade Purchase 2010; SAGE Deep Backfile Upgrade Purchase 2011; SAGE Deep Backfile Upgrade Purchase 2012; SAGE Deep Backfile Upgrade Purchase 2013; SAGE Deep Backfile Upgrade Purchase 2014; SAGE Deep Backfile Upgrade Purchase 2015; SAGE Deep Backfile Upgrade Purchase 2016; SAGE Deep Backfile Upgrade Purchase 2017; SAGE Psychology Subject Collection Backfile Purchase; Taylor &amp; Francis online monographs (EBS) purchased</x:t>
         </x:is>
       </x:c>
       <x:c r="C506" s="9" t="inlineStr">
@@ -14765,7 +14765,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27aecb3ab50d40b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R388488dcf290403d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17261,7 +17261,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442a36a7096d49d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafdefb6fa4a84725"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
improving symmetry of the saved column and filter flow
</commit_message>
<xml_diff>
--- a/output/saved_column_review.xlsx
+++ b/output/saved_column_review.xlsx
@@ -19321,46 +19321,51 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>saved_column_object_index</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>catalog_index</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>saved_column_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>column_type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>table_heading</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>column_heading</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>base_formula</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>rule_count</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>original_path</t>
         </is>
@@ -19370,35 +19375,38 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Electronic - Count of Electronic Holdings</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Calculated column</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Holdings</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>COUNT(DISTINCT "Portfolio"."Portfolio Id")</t>
         </is>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - Count of Electronic Holdings</t>
         </is>
@@ -19408,35 +19416,38 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Electronic - Count of Electronic Titles</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Calculated column</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Bibliographic Details</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Titles</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>COUNT(DISTINCT "Bibliographic Details"."MMS Id")</t>
         </is>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - Count of Electronic Titles</t>
         </is>
@@ -19444,37 +19455,40 @@
     </row>
     <row r="4">
       <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
         <v>7</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Electronic - Global Stats Electronic included/excluded designator</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Electronic Collection</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>eResources include/exclude designator</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>"Electronic Collection"."Electronic Collection Interface Name"</t>
         </is>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>34</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - Global Stats Electronic included/excluded designator</t>
         </is>
@@ -19482,37 +19496,40 @@
     </row>
     <row r="5">
       <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
         <v>24</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Electronic - Global Stats Electronic Library Categories</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>UCOP Stats</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>eResources Library Stats Category</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>"Portfolio Library Unit"."Library Name"</t>
         </is>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>5</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - Global Stats Electronic Library Categories</t>
         </is>
@@ -19520,37 +19537,40 @@
     </row>
     <row r="6">
       <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
         <v>57</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Electronic - UCB eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>UCB eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>4</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCB eResources Managed By designator</t>
         </is>
@@ -19558,37 +19578,40 @@
     </row>
     <row r="7">
       <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
         <v>100</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Electronic - UCD eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>UCD eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>4</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCD eResources Managed By designator</t>
         </is>
@@ -19596,37 +19619,40 @@
     </row>
     <row r="8">
       <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
         <v>114</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Electronic - UCI eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>UCI eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>4</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCI eResources Managed By designator</t>
         </is>
@@ -19634,37 +19660,40 @@
     </row>
     <row r="9">
       <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
         <v>143</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Electronic - UCLA eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>UCLA eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>4</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCLA eResources Managed By designator</t>
         </is>
@@ -19672,37 +19701,40 @@
     </row>
     <row r="10">
       <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
         <v>165</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Electronic - UCM eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>UCM eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>4</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCM eResources Managed By designator</t>
         </is>
@@ -19710,37 +19742,40 @@
     </row>
     <row r="11">
       <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
         <v>179</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Electronic - UCR eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>UCR eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>4</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCR eResources Managed By designator</t>
         </is>
@@ -19748,37 +19783,40 @@
     </row>
     <row r="12">
       <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
         <v>195</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Electronic - UCSB eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>UCSB eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>4</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCSB eResources Managed By designator</t>
         </is>
@@ -19786,37 +19824,40 @@
     </row>
     <row r="13">
       <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
         <v>200</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Electronic - UCSC eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>UCSC eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>4</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCSC eResources Managed By designator</t>
         </is>
@@ -19824,37 +19865,40 @@
     </row>
     <row r="14">
       <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
         <v>209</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Electronic - UCSD eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>UCSD eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>4</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic - UCSD eResources Managed By designator</t>
         </is>
@@ -19862,37 +19906,40 @@
     </row>
     <row r="15">
       <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
         <v>218</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Electronic UCSF eResources Managed By designator</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>UCSF eResources Managed By designator</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>4</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Electronic UCSF eResources Managed By designator</t>
         </is>
@@ -19900,37 +19947,40 @@
     </row>
     <row r="16">
       <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
         <v>222</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Fulfillment - Alma User Group</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Calculated column</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Alma User Group</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>1</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - Alma User Group</t>
         </is>
@@ -19938,37 +19988,40 @@
     </row>
     <row r="17">
       <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
         <v>224</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Fulfillment - Fulfillment Institution</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Fulfillment Institution</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>13</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - Fulfillment Institution</t>
         </is>
@@ -19976,37 +20029,40 @@
     </row>
     <row r="18">
       <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
         <v>229</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Fulfillment - FY 2025-26 Loans (Not In House)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Calculated column</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Loan</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>FY 2025-26 Loans (Not In House)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>"Loan"."Loans (Not In House)"</t>
         </is>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>1</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - FY 2025-26 Loans (Not In House)</t>
         </is>
@@ -20014,37 +20070,40 @@
     </row>
     <row r="19">
       <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
         <v>233</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Fulfillment - UCB Check-Out Type</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>UCB Check-Out Type</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>6</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCB Check-Out Type</t>
         </is>
@@ -20052,37 +20111,40 @@
     </row>
     <row r="20">
       <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
         <v>235</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Fulfillment - UCB User Group</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>UCB User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>12</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCB User Group</t>
         </is>
@@ -20090,37 +20152,40 @@
     </row>
     <row r="21">
       <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
         <v>239</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Fulfillment - UCD Check-Out Type</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>UCD Check-Out Type</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>6</v>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCD Check-Out Type</t>
         </is>
@@ -20128,37 +20193,40 @@
     </row>
     <row r="22">
       <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
         <v>240</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Fulfillment - UCD User Group</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>UCD User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>11</v>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCD User Group</t>
         </is>
@@ -20166,37 +20234,40 @@
     </row>
     <row r="23">
       <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
         <v>242</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Fulfillment - UCI Check-Out Type</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>UCI Check-Out Type</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>8</v>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCI Check-Out Type</t>
         </is>
@@ -20204,37 +20275,40 @@
     </row>
     <row r="24">
       <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
         <v>244</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Fulfillment - UCI User Group</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>UCI User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>11</v>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCI User Group</t>
         </is>
@@ -20242,37 +20316,40 @@
     </row>
     <row r="25">
       <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
         <v>246</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Fulfillment - UCLA Check-Out Type</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>UCLA Check-Out Type</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>7</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCLA Check-Out Type</t>
         </is>
@@ -20280,37 +20357,40 @@
     </row>
     <row r="26">
       <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
         <v>249</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Fulfillment - UCLA User Group</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>UCLA User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>11</v>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCLA User Group</t>
         </is>
@@ -20318,37 +20398,40 @@
     </row>
     <row r="27">
       <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
         <v>250</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Fulfillment - UCM Check-Out Type</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>UCM Check-Out Type</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G27">
+      <c r="H27">
         <v>5</v>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCM Check-Out Type</t>
         </is>
@@ -20356,37 +20439,40 @@
     </row>
     <row r="28">
       <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
         <v>251</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Fulfillment - UCM User Group</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>UCM User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G28">
+      <c r="H28">
         <v>9</v>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCM User Group</t>
         </is>
@@ -20394,37 +20480,40 @@
     </row>
     <row r="29">
       <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
         <v>252</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Fulfillment - UCR Check-Out Type</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>UCR Check-Out Type</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>7</v>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCR Check-Out Type</t>
         </is>
@@ -20432,37 +20521,40 @@
     </row>
     <row r="30">
       <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
         <v>253</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Fulfillment - UCR User Group</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>UCR User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G30">
+      <c r="H30">
         <v>11</v>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCR User Group</t>
         </is>
@@ -20470,37 +20562,40 @@
     </row>
     <row r="31">
       <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
         <v>254</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Fulfillment - UCSB Check-Out Type</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>UCSB Check-Out Type</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G31">
+      <c r="H31">
         <v>8</v>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSB Check-Out Type</t>
         </is>
@@ -20508,37 +20603,40 @@
     </row>
     <row r="32">
       <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
         <v>255</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Fulfillment - UCSB User Group</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>UCSB User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G32">
+      <c r="H32">
         <v>11</v>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSB User Group</t>
         </is>
@@ -20546,37 +20644,40 @@
     </row>
     <row r="33">
       <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
         <v>256</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Fulfillment - UCSC Check-Out Type</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>UCSC Check-Out Type</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G33">
+      <c r="H33">
         <v>7</v>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSC Check-Out Type</t>
         </is>
@@ -20584,37 +20685,40 @@
     </row>
     <row r="34">
       <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
         <v>257</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Fulfillment - UCSC User Group</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>UCSC User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G34">
+      <c r="H34">
         <v>10</v>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSC User Group</t>
         </is>
@@ -20622,37 +20726,40 @@
     </row>
     <row r="35">
       <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
         <v>258</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Fulfillment - UCSD Check-Out Type</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>UCSD Check-Out Type</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G35">
+      <c r="H35">
         <v>6</v>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSD Check-Out Type</t>
         </is>
@@ -20660,37 +20767,40 @@
     </row>
     <row r="36">
       <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
         <v>259</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Fulfillment - UCSD User Group</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>UCSD User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G36">
+      <c r="H36">
         <v>11</v>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSD User Group</t>
         </is>
@@ -20698,37 +20808,40 @@
     </row>
     <row r="37">
       <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
         <v>260</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Fulfillment - UCSF Check-Out Type</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Item Location at Time of Loan</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>UCSF Check-Out Type</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>"Item Location at Time of Loan"."Location Code"</t>
         </is>
       </c>
-      <c r="G37">
+      <c r="H37">
         <v>6</v>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSF Check-Out Type</t>
         </is>
@@ -20736,37 +20849,40 @@
     </row>
     <row r="38">
       <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
         <v>261</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Fulfillment - UCSF User Group</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Borrower Details</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>UCSF User Group (for reporting)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>"Borrower Details"."User Group"</t>
         </is>
       </c>
-      <c r="G38">
+      <c r="H38">
         <v>6</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Fulfillment - UCSF User Group</t>
         </is>
@@ -20774,37 +20890,40 @@
     </row>
     <row r="39">
       <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
         <v>262</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Physical - Count of Physical Holdings</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Calculated column</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Physical Item Details</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Holdings</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>COUNT(DISTINCT "Physical Item Details"."Physical Item Id")</t>
         </is>
       </c>
-      <c r="G39">
+      <c r="H39">
         <v>1</v>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - Count of Physical Holdings</t>
         </is>
@@ -20812,37 +20931,40 @@
     </row>
     <row r="40">
       <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
         <v>263</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Physical - Count of Physical Titles</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Calculated column</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Bibliographic Details</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Titles</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>COUNT(DISTINCT "Bibliographic Details"."MMS ID")</t>
         </is>
       </c>
-      <c r="G40">
+      <c r="H40">
         <v>1</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - Count of Physical Titles</t>
         </is>
@@ -20850,37 +20972,40 @@
     </row>
     <row r="41">
       <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
         <v>265</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Physical - Holdings Added Year</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Item Creation Date</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Holdings Added Year</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>"Item Creation Date"."Item Creation Date"</t>
         </is>
       </c>
-      <c r="G41">
+      <c r="H41">
         <v>2</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - Holdings Added Year</t>
         </is>
@@ -20888,37 +21013,40 @@
     </row>
     <row r="42">
       <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
         <v>266</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Physical - SLF Depositor</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>SLF Depositor</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G42">
+      <c r="H42">
         <v>33</v>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - SLF Depositor</t>
         </is>
@@ -20926,37 +21054,40 @@
     </row>
     <row r="43">
       <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
         <v>269</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Physical - Systemwide Library Facility</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Systemwide Library Facility</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G43">
+      <c r="H43">
         <v>3</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - Systemwide Library Facility</t>
         </is>
@@ -20964,37 +21095,40 @@
     </row>
     <row r="44">
       <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
         <v>270</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Physical - UCB Library Stats Category</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>UCB Library Stats Category</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G44">
+      <c r="H44">
         <v>13</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCB Library Stats Category</t>
         </is>
@@ -21002,37 +21136,40 @@
     </row>
     <row r="45">
       <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
         <v>273</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Physical - UCB SLF/Campus designator</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>UCB SLF/campus designator</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G45">
+      <c r="H45">
         <v>8</v>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCB SLF/Campus designator</t>
         </is>
@@ -21040,37 +21177,40 @@
     </row>
     <row r="46">
       <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
         <v>274</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Physical - UCD Library Stats Category</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>UCD Library Stats Category</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G46">
+      <c r="H46">
         <v>11</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCD Library Stats Category</t>
         </is>
@@ -21078,37 +21218,40 @@
     </row>
     <row r="47">
       <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
         <v>276</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Physical - UCD SLF/campus designator</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>UCD SLF/campus designator</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G47">
+      <c r="H47">
         <v>7</v>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCD SLF/campus designator</t>
         </is>
@@ -21116,37 +21259,40 @@
     </row>
     <row r="48">
       <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
         <v>277</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Physical - UCI Library Stats Category</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>UCI Library Stats Category</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G48">
+      <c r="H48">
         <v>8</v>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCI Library Stats Category</t>
         </is>
@@ -21154,37 +21300,40 @@
     </row>
     <row r="49">
       <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
         <v>280</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Physical - UCI SLF/campus designator</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>UCI SLF/campus designator</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G49">
+      <c r="H49">
         <v>5</v>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCI SLF/campus designator</t>
         </is>
@@ -21192,37 +21341,40 @@
     </row>
     <row r="50">
       <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
         <v>281</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Physical - UCLA Library Stats Category</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>UCLA Library Stats Category</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G50">
+      <c r="H50">
         <v>13</v>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCLA Library Stats Category</t>
         </is>
@@ -21230,37 +21382,40 @@
     </row>
     <row r="51">
       <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
         <v>284</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Physical - UCLA SLF/campus designator</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>UCLA SLF/campus designator</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G51">
+      <c r="H51">
         <v>6</v>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCLA SLF/campus designator</t>
         </is>
@@ -21268,37 +21423,40 @@
     </row>
     <row r="52">
       <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
         <v>285</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>Physical - UCM Library Stats Category</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>UCM Library Stats Category</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>"Location"."Location Code"</t>
         </is>
       </c>
-      <c r="G52">
+      <c r="H52">
         <v>5</v>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCM Library Stats Category</t>
         </is>
@@ -21306,37 +21464,40 @@
     </row>
     <row r="53">
       <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
         <v>286</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>Physical - UCM SLF/campus designator</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>UCM SLF/campus designator</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G53">
+      <c r="H53">
         <v>3</v>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCM SLF/campus designator</t>
         </is>
@@ -21344,37 +21505,40 @@
     </row>
     <row r="54">
       <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
         <v>287</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>Physical - UCR Library Stats Category</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>UCR Library Stats Category</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G54">
+      <c r="H54">
         <v>8</v>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCR Library Stats Category</t>
         </is>
@@ -21382,37 +21546,40 @@
     </row>
     <row r="55">
       <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
         <v>290</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Physical - UCR SLF/campus designator</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>UCR SLF/campus designator</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G55">
+      <c r="H55">
         <v>5</v>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCR SLF/campus designator</t>
         </is>
@@ -21420,37 +21587,40 @@
     </row>
     <row r="56">
       <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
         <v>291</v>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Physical - UCSB Library Stats Category</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>UCSB Library Stats Category</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G56">
+      <c r="H56">
         <v>7</v>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSB Library Stats Category</t>
         </is>
@@ -21458,37 +21628,40 @@
     </row>
     <row r="57">
       <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
         <v>293</v>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Physical - UCSB SLF/campus designator</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>UCSB SLF/campus designator</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G57">
+      <c r="H57">
         <v>5</v>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSB SLF/campus designator</t>
         </is>
@@ -21496,37 +21669,40 @@
     </row>
     <row r="58">
       <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
         <v>294</v>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>Physical - UCSC Library Stats Category</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>UCSC Library Stats Category</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G58">
+      <c r="H58">
         <v>6</v>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSC Library Stats Category</t>
         </is>
@@ -21534,37 +21710,40 @@
     </row>
     <row r="59">
       <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
         <v>297</v>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Physical - UCSC SLF/campus designator</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>UCSC SLF/campus designator</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G59">
+      <c r="H59">
         <v>5</v>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSC SLF/campus designator</t>
         </is>
@@ -21572,37 +21751,40 @@
     </row>
     <row r="60">
       <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
         <v>298</v>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Physical - UCSD Library Stats Category</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>UCSD Library Stats Category</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G60">
+      <c r="H60">
         <v>6</v>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSD Library Stats Category</t>
         </is>
@@ -21610,37 +21792,40 @@
     </row>
     <row r="61">
       <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
         <v>301</v>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Physical - UCSD SLF/campus designator</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>UCSD SLF/campus designator</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G61">
+      <c r="H61">
         <v>5</v>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSD SLF/campus designator</t>
         </is>
@@ -21648,37 +21833,40 @@
     </row>
     <row r="62">
       <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
         <v>302</v>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Physical - UCSF Library Stats Category</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>UCSF Library Stats Category</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>"Location"."Library Code"</t>
         </is>
       </c>
-      <c r="G62">
+      <c r="H62">
         <v>6</v>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSF Library Stats Category</t>
         </is>
@@ -21686,37 +21874,40 @@
     </row>
     <row r="63">
       <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
         <v>304</v>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>Physical - UCSF SLF/campus designator</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>UCSF SLF/campus designator</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>"Institution"."Institution Name"</t>
         </is>
       </c>
-      <c r="G63">
+      <c r="H63">
         <v>5</v>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/Physical - UCSF SLF/campus designator</t>
         </is>
@@ -21724,37 +21915,40 @@
     </row>
     <row r="64">
       <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
         <v>305</v>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>RM Building - UCB</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>Building</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>"Location"."Location Code"</t>
         </is>
       </c>
-      <c r="G64">
+      <c r="H64">
         <v>33</v>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/RM Building - UCB</t>
         </is>
@@ -21762,37 +21956,40 @@
     </row>
     <row r="65">
       <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
         <v>308</v>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>zzBACKUP Electronic - Global Stats Electronic included/excluded designator</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Binned column</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>UCOP Stats</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>eResources include/exclude designator</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>"Electronic Collection"."Electronic Collection Public Name"</t>
         </is>
       </c>
-      <c r="G65">
+      <c r="H65">
         <v>36</v>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>/shared/University of California System 01UCS_NETWORK/Reports/Local Requests/Annual Statistic Reports/Annual Stats FY 2025-2026/zzBACKUP Electronic - Global Stats Electronic included/excluded designator</t>
         </is>

</xml_diff>